<commit_message>
feat: Add role-based user deletion and refactor wipe-firestore.js
- Add selective user deletion by role (teachers, admins, or both)
- Implement universal confirmation prompt for all deletion operations
- Consolidate confirmation logic into reusable confirmAction() function
- Eliminate redundant readline interfaces and duplicate code
- Streamline async/await patterns for better maintainability
- Maintain safety with mandatory confirmation for all destructive operations

Usage: node wipe-firestore.js users
Then select: 1 (teachers only), 2 (admins only), or 3 (both)
</commit_message>
<xml_diff>
--- a/data/raw/educators-list-uncleaned.xlsx
+++ b/data/raw/educators-list-uncleaned.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="149">
   <si>
     <t>Location</t>
   </si>
@@ -28,7 +28,7 @@
     <t>HSR</t>
   </si>
   <si>
-    <t>All Stars</t>
+    <t>Adolescent</t>
   </si>
   <si>
     <t>Rahul Raghavan</t>
@@ -97,7 +97,7 @@
         <color theme="1"/>
         <sz val="11.0"/>
       </rPr>
-      <t xml:space="preserve"> All Stars/Power/Amazing/Plumeria/Perinwinkle/Gulmohar 
+      <t xml:space="preserve"> Adolescent/Power/Amazing/Plumeria/Perinwinkle/Gulmohar 
 </t>
     </r>
     <r>
@@ -140,7 +140,7 @@
         <color theme="1"/>
         <sz val="11.0"/>
       </rPr>
-      <t xml:space="preserve"> All Stars/Power/Amazing/Plumeria/Perinwinkle/Gulmohar 
+      <t xml:space="preserve"> Adolescent/Power/Amazing/Plumeria/Perinwinkle/Gulmohar 
 </t>
     </r>
     <r>
@@ -183,7 +183,7 @@
         <color theme="1"/>
         <sz val="11.0"/>
       </rPr>
-      <t xml:space="preserve"> All Stars/Power/Amazing
+      <t xml:space="preserve"> Adolescent/Power/Amazing
 </t>
     </r>
     <r>
@@ -265,7 +265,7 @@
     <t>sandhya@pepschoolv2.com</t>
   </si>
   <si>
-    <t>Amazing/Power/All Stars</t>
+    <t>Amazing/Power/Adolescent</t>
   </si>
   <si>
     <t>Sonika Rana</t>
@@ -507,6 +507,60 @@
   <si>
     <t>amirtha.lakshmi@ribbons.education</t>
   </si>
+  <si>
+    <t xml:space="preserve">Hyderabad </t>
+  </si>
+  <si>
+    <t>Primary 1</t>
+  </si>
+  <si>
+    <t>Archana Dodethker</t>
+  </si>
+  <si>
+    <t>archanadodethker@pepschoolv2.com</t>
+  </si>
+  <si>
+    <t>Padmavati</t>
+  </si>
+  <si>
+    <t>padmavati@pepschoolv2.com</t>
+  </si>
+  <si>
+    <t>Rimsha</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>Primary 2</t>
+  </si>
+  <si>
+    <t>Vanitha</t>
+  </si>
+  <si>
+    <t>vanitha@pepschoolv2.com</t>
+  </si>
+  <si>
+    <t>Padmaja</t>
+  </si>
+  <si>
+    <t>padmaja@pepschoolv2.com</t>
+  </si>
+  <si>
+    <t>Priyanka Tijare</t>
+  </si>
+  <si>
+    <t>priyanka@pepschoolv2.com</t>
+  </si>
+  <si>
+    <t>Toddler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kauser </t>
+  </si>
+  <si>
+    <t>kauser@pepschoolv2.com</t>
+  </si>
 </sst>
 </file>
 
@@ -599,10 +653,10 @@
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
+      <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
@@ -834,7 +888,8 @@
   <cols>
     <col customWidth="1" min="2" max="2" width="19.75"/>
     <col customWidth="1" min="3" max="3" width="61.75"/>
-    <col customWidth="1" min="4" max="5" width="31.13"/>
+    <col customWidth="1" min="4" max="4" width="31.13"/>
+    <col customWidth="1" min="5" max="5" width="34.75"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -970,13 +1025,13 @@
       <c r="B5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="6" t="s">
         <v>9</v>
       </c>
       <c r="F5" s="1"/>
@@ -1006,13 +1061,13 @@
       <c r="B6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="7" t="s">
         <v>11</v>
       </c>
       <c r="F6" s="1"/>
@@ -1042,13 +1097,13 @@
       <c r="B7" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="7" t="s">
         <v>13</v>
       </c>
       <c r="F7" s="1"/>
@@ -1078,13 +1133,13 @@
       <c r="B8" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="7" t="s">
         <v>15</v>
       </c>
       <c r="F8" s="1"/>
@@ -1114,7 +1169,7 @@
       <c r="B9" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="5" t="s">
         <v>5</v>
       </c>
       <c r="D9" s="5" t="s">
@@ -1150,7 +1205,7 @@
       <c r="B10" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="5" t="s">
         <v>5</v>
       </c>
       <c r="D10" s="5" t="s">
@@ -1186,7 +1241,7 @@
       <c r="B11" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="5" t="s">
         <v>5</v>
       </c>
       <c r="D11" s="5" t="s">
@@ -1333,10 +1388,10 @@
       <c r="C15" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="E15" s="7" t="s">
         <v>33</v>
       </c>
       <c r="F15" s="1"/>
@@ -1369,10 +1424,10 @@
       <c r="C16" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="6" t="s">
         <v>35</v>
       </c>
       <c r="F16" s="1"/>
@@ -1405,10 +1460,10 @@
       <c r="C17" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="D17" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E17" s="7" t="s">
         <v>37</v>
       </c>
       <c r="F17" s="1"/>
@@ -1441,10 +1496,10 @@
       <c r="C18" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F18" s="1"/>
@@ -1477,10 +1532,10 @@
       <c r="C19" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D19" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="E19" s="7" t="s">
         <v>42</v>
       </c>
       <c r="F19" s="1"/>
@@ -1513,10 +1568,10 @@
       <c r="C20" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="D20" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="E20" s="6" t="s">
         <v>44</v>
       </c>
       <c r="F20" s="1"/>
@@ -1549,10 +1604,10 @@
       <c r="C21" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="E21" s="7" t="s">
         <v>47</v>
       </c>
       <c r="F21" s="1"/>
@@ -1585,10 +1640,10 @@
       <c r="C22" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="E22" s="7" t="s">
         <v>49</v>
       </c>
       <c r="F22" s="1"/>
@@ -1621,10 +1676,10 @@
       <c r="C23" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D23" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="E23" s="7" t="s">
         <v>52</v>
       </c>
       <c r="F23" s="1"/>
@@ -1657,10 +1712,10 @@
       <c r="C24" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="D24" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="E24" s="7" t="s">
         <v>55</v>
       </c>
       <c r="F24" s="1"/>
@@ -1693,10 +1748,10 @@
       <c r="C25" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="D25" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="E25" s="6" t="s">
+      <c r="E25" s="7" t="s">
         <v>57</v>
       </c>
       <c r="F25" s="1"/>
@@ -1729,10 +1784,10 @@
       <c r="C26" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D26" s="6" t="s">
+      <c r="D26" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="E26" s="6" t="s">
+      <c r="E26" s="7" t="s">
         <v>59</v>
       </c>
       <c r="F26" s="1"/>
@@ -1765,10 +1820,10 @@
       <c r="C27" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="D27" s="6" t="s">
+      <c r="D27" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="E27" s="6" t="s">
+      <c r="E27" s="7" t="s">
         <v>62</v>
       </c>
       <c r="F27" s="1"/>
@@ -1801,10 +1856,10 @@
       <c r="C28" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="D28" s="6" t="s">
+      <c r="D28" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="E28" s="6" t="s">
+      <c r="E28" s="7" t="s">
         <v>64</v>
       </c>
       <c r="F28" s="1"/>
@@ -1837,10 +1892,10 @@
       <c r="C29" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="D29" s="7" t="s">
+      <c r="D29" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="E29" s="7" t="s">
         <v>66</v>
       </c>
       <c r="F29" s="1"/>
@@ -1873,10 +1928,10 @@
       <c r="C30" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="D30" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="E30" s="6" t="s">
+      <c r="E30" s="7" t="s">
         <v>69</v>
       </c>
       <c r="F30" s="1"/>
@@ -1909,10 +1964,10 @@
       <c r="C31" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="D31" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="E31" s="6" t="s">
+      <c r="E31" s="7" t="s">
         <v>71</v>
       </c>
       <c r="F31" s="1"/>
@@ -1945,10 +2000,10 @@
       <c r="C32" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D32" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="E32" s="6" t="s">
+      <c r="E32" s="7" t="s">
         <v>74</v>
       </c>
       <c r="F32" s="1"/>
@@ -1981,10 +2036,10 @@
       <c r="C33" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="D33" s="6" t="s">
+      <c r="D33" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="E33" s="6" t="s">
+      <c r="E33" s="7" t="s">
         <v>77</v>
       </c>
       <c r="F33" s="1"/>
@@ -2017,10 +2072,10 @@
       <c r="C34" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="D34" s="7" t="s">
+      <c r="D34" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="E34" s="6" t="s">
+      <c r="E34" s="7" t="s">
         <v>80</v>
       </c>
       <c r="F34" s="1"/>
@@ -2053,10 +2108,10 @@
       <c r="C35" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="D35" s="7" t="s">
+      <c r="D35" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="E35" s="6" t="s">
+      <c r="E35" s="7" t="s">
         <v>82</v>
       </c>
       <c r="F35" s="1"/>
@@ -2089,10 +2144,10 @@
       <c r="C36" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="D36" s="6" t="s">
+      <c r="D36" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="E36" s="6" t="s">
+      <c r="E36" s="7" t="s">
         <v>84</v>
       </c>
       <c r="F36" s="1"/>
@@ -2125,10 +2180,10 @@
       <c r="C37" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="D37" s="6" t="s">
+      <c r="D37" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="E37" s="6" t="s">
+      <c r="E37" s="7" t="s">
         <v>86</v>
       </c>
       <c r="F37" s="1"/>
@@ -2731,10 +2786,18 @@
     </row>
     <row r="54">
       <c r="A54" s="1"/>
-      <c r="B54" s="2"/>
-      <c r="C54" s="3"/>
-      <c r="D54" s="3"/>
-      <c r="E54" s="3"/>
+      <c r="B54" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C54" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="D54" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E54" s="5" t="s">
+        <v>134</v>
+      </c>
       <c r="F54" s="1"/>
       <c r="G54" s="1"/>
       <c r="H54" s="1"/>
@@ -2759,10 +2822,18 @@
     </row>
     <row r="55">
       <c r="A55" s="1"/>
-      <c r="B55" s="2"/>
-      <c r="C55" s="3"/>
-      <c r="D55" s="3"/>
-      <c r="E55" s="3"/>
+      <c r="B55" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C55" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="D55" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="E55" s="5" t="s">
+        <v>136</v>
+      </c>
       <c r="F55" s="1"/>
       <c r="G55" s="1"/>
       <c r="H55" s="1"/>
@@ -2787,10 +2858,18 @@
     </row>
     <row r="56">
       <c r="A56" s="1"/>
-      <c r="B56" s="2"/>
-      <c r="C56" s="3"/>
-      <c r="D56" s="3"/>
-      <c r="E56" s="3"/>
+      <c r="B56" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="D56" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="E56" s="5" t="s">
+        <v>138</v>
+      </c>
       <c r="F56" s="1"/>
       <c r="G56" s="1"/>
       <c r="H56" s="1"/>
@@ -2815,10 +2894,18 @@
     </row>
     <row r="57">
       <c r="A57" s="1"/>
-      <c r="B57" s="2"/>
-      <c r="C57" s="3"/>
-      <c r="D57" s="3"/>
-      <c r="E57" s="3"/>
+      <c r="B57" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C57" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="D57" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="E57" s="5" t="s">
+        <v>141</v>
+      </c>
       <c r="F57" s="1"/>
       <c r="G57" s="1"/>
       <c r="H57" s="1"/>
@@ -2843,10 +2930,18 @@
     </row>
     <row r="58">
       <c r="A58" s="1"/>
-      <c r="B58" s="2"/>
-      <c r="C58" s="3"/>
-      <c r="D58" s="3"/>
-      <c r="E58" s="3"/>
+      <c r="B58" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C58" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="D58" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="E58" s="5" t="s">
+        <v>143</v>
+      </c>
       <c r="F58" s="1"/>
       <c r="G58" s="1"/>
       <c r="H58" s="1"/>
@@ -2871,10 +2966,18 @@
     </row>
     <row r="59">
       <c r="A59" s="1"/>
-      <c r="B59" s="2"/>
-      <c r="C59" s="3"/>
-      <c r="D59" s="3"/>
-      <c r="E59" s="3"/>
+      <c r="B59" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="D59" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="E59" s="5" t="s">
+        <v>145</v>
+      </c>
       <c r="F59" s="1"/>
       <c r="G59" s="1"/>
       <c r="H59" s="1"/>
@@ -2899,10 +3002,18 @@
     </row>
     <row r="60">
       <c r="A60" s="1"/>
-      <c r="B60" s="2"/>
-      <c r="C60" s="3"/>
-      <c r="D60" s="3"/>
-      <c r="E60" s="3"/>
+      <c r="B60" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C60" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="D60" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="E60" s="5" t="s">
+        <v>148</v>
+      </c>
       <c r="F60" s="1"/>
       <c r="G60" s="1"/>
       <c r="H60" s="1"/>

</xml_diff>